<commit_message>
feat(planejamento): harmonizacao 3 vias CPM/LOB/Takt, auditoria multi-eixo e motores multiobra puros
- Harmoniza rigorosamente os 3 cronogramas da OBRA_TMULT em 178 dias úteis (término 26/04/2027) com zero gap
- Corrige sequência do Portão 4 (emassamento/1ª demão -> louças/luminárias -> pintura final)
- Cria motor universal scripts/auditar_cronogramas.py com validação dos 5 eixos matemáticos
- Unifica a esteira takt universal em scripts/gerar_programacao_curto_prazo_takt.py com suporte a --obra
- Move scripts legados/específicos para scripts/_legado_tmult e scripts/_obsoletos, garantindo scripts/ 100% multiobra
- Adiciona componente executivo Gantt (GanttExecutivo.tsx) e abas integradas no Dashboard Next.js
- Atualiza documentação de governança: README.md (23 motores), agents.md, README_COMO_CRIAR_NOVA_OBRA.md, SKILL_GESTAO_16 e RELATORIO_PLANEJAMENTO_BASELINE_TMULT.md
</commit_message>
<xml_diff>
--- a/projetos/OBRA_TMULT/03_PLANEJAMENTO_E_CRONOGRAMA/CRONOGRAMA_FISICO_FINANCEIRO_TMULT.xlsx
+++ b/projetos/OBRA_TMULT/03_PLANEJAMENTO_E_CRONOGRAMA/CRONOGRAMA_FISICO_FINANCEIRO_TMULT.xlsx
@@ -821,16 +821,16 @@
         </is>
       </c>
       <c r="C8" s="5" t="n">
-        <v>366373.12</v>
+        <v>347328.2</v>
       </c>
       <c r="D8" s="6" t="n">
-        <v>0.220605395734301</v>
+        <v>0.2091378183276176</v>
       </c>
       <c r="E8" s="5" t="n">
-        <v>807710.99</v>
+        <v>788666.0699999999</v>
       </c>
       <c r="F8" s="6" t="n">
-        <v>0.4863495514842739</v>
+        <v>0.4748819740775905</v>
       </c>
       <c r="G8" s="6" t="n">
         <v>0.541</v>
@@ -843,16 +843,16 @@
         </is>
       </c>
       <c r="C9" s="8" t="n">
-        <v>245681.39</v>
+        <v>251786.96</v>
       </c>
       <c r="D9" s="9" t="n">
-        <v>0.1479329058461034</v>
+        <v>0.1516092718579808</v>
       </c>
       <c r="E9" s="8" t="n">
-        <v>1053392.38</v>
+        <v>1040453.03</v>
       </c>
       <c r="F9" s="9" t="n">
-        <v>0.6342824573303772</v>
+        <v>0.6264912459355713</v>
       </c>
       <c r="G9" s="9" t="n">
         <v>0.6984999999999999</v>
@@ -865,10 +865,10 @@
         </is>
       </c>
       <c r="C10" s="5" t="n">
-        <v>320416.9</v>
+        <v>333356.25</v>
       </c>
       <c r="D10" s="6" t="n">
-        <v>0.1929336328616519</v>
+        <v>0.200724844256458</v>
       </c>
       <c r="E10" s="5" t="n">
         <v>1373809.28</v>
@@ -6088,22 +6088,22 @@
         <v>0</v>
       </c>
       <c r="L75" s="6" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M75" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="N75" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="O75" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="P75" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q75" s="5" t="n">
         <v>8420.219999999999</v>
-      </c>
-      <c r="N75" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="O75" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="P75" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q75" s="5" t="n">
-        <v>0</v>
       </c>
       <c r="R75" s="6" t="n">
         <v>0</v>
@@ -6159,22 +6159,22 @@
         <v>0</v>
       </c>
       <c r="L76" s="9" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M76" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="N76" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="O76" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="P76" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q76" s="8" t="n">
         <v>4519.13</v>
-      </c>
-      <c r="N76" s="9" t="n">
-        <v>0</v>
-      </c>
-      <c r="O76" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="P76" s="9" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q76" s="8" t="n">
-        <v>0</v>
       </c>
       <c r="R76" s="9" t="n">
         <v>0</v>
@@ -6230,16 +6230,16 @@
         <v>0</v>
       </c>
       <c r="L77" s="6" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M77" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="N77" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="O77" s="5" t="n">
         <v>5611.09</v>
-      </c>
-      <c r="N77" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="O77" s="5" t="n">
-        <v>0</v>
       </c>
       <c r="P77" s="6" t="n">
         <v>0</v>
@@ -6301,16 +6301,16 @@
         <v>0</v>
       </c>
       <c r="L78" s="9" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M78" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="N78" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="O78" s="8" t="n">
         <v>494.48</v>
-      </c>
-      <c r="N78" s="9" t="n">
-        <v>0</v>
-      </c>
-      <c r="O78" s="8" t="n">
-        <v>0</v>
       </c>
       <c r="P78" s="9" t="n">
         <v>0</v>

</xml_diff>